<commit_message>
South African total alkalinity
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2531" uniqueCount="1307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2567" uniqueCount="1332">
   <si>
     <t>GEMS Station Number</t>
   </si>
@@ -3819,16 +3819,28 @@
     <t>Parameter Description</t>
   </si>
   <si>
-    <t>EC</t>
-  </si>
-  <si>
-    <t>Electrical Conductance</t>
-  </si>
-  <si>
-    <t>/Chemical/Inorganic/Bulk Property</t>
-  </si>
-  <si>
-    <t>Measure of the ability of water to carry an electric current.</t>
+    <t>Alk-Tot</t>
+  </si>
+  <si>
+    <t>Alkalinity</t>
+  </si>
+  <si>
+    <t>Total Alkalinity</t>
+  </si>
+  <si>
+    <t>/Chemical/Inorganic/Non-Metal</t>
+  </si>
+  <si>
+    <t>207-439-9</t>
+  </si>
+  <si>
+    <t>471-34-1</t>
+  </si>
+  <si>
+    <t>3311</t>
+  </si>
+  <si>
+    <t>Acid-neutralizing capacity of sample at the point, when all Carbonate (CO32-) and Bicarbonate (HCO3-) have reacted, reported as mg CaCO3/L.</t>
   </si>
   <si>
     <t>Analysis Method Code</t>
@@ -3852,67 +3864,106 @@
     <t>Method Description</t>
   </si>
   <si>
-    <t>EC-CAL</t>
-  </si>
-  <si>
-    <t>EC-CND</t>
-  </si>
-  <si>
-    <t>EC-CND-FLD</t>
-  </si>
-  <si>
-    <t>EC-CND-Ni</t>
-  </si>
-  <si>
-    <t>EC-CND-Pt</t>
-  </si>
-  <si>
-    <t>EC-CND-Pt-AMB</t>
-  </si>
-  <si>
-    <t>FCS-CND</t>
-  </si>
-  <si>
-    <t>µS/cm</t>
-  </si>
-  <si>
-    <t>Calculated Theoretical Conductivity</t>
-  </si>
-  <si>
-    <t>Electrometer at 20°C</t>
-  </si>
-  <si>
-    <t>Conductivity Meter - Field measurement</t>
-  </si>
-  <si>
-    <t>Conductivity-Temperature Meter using Nickel Electrode (at 25°C)</t>
-  </si>
-  <si>
-    <t>Laboratory Method using Platinum Electrode (at 25°C)</t>
-  </si>
-  <si>
-    <t>Laboratory Method using Platinum Electrode (at Ambient Temperature)</t>
-  </si>
-  <si>
-    <t>Field Conductivity Sensor</t>
-  </si>
-  <si>
-    <t>Calculation</t>
-  </si>
-  <si>
-    <t>Electrochemical Analysis</t>
-  </si>
-  <si>
-    <t>ENV 2355</t>
-  </si>
-  <si>
-    <t>ENV 33</t>
-  </si>
-  <si>
-    <t>SM 2510 B</t>
-  </si>
-  <si>
-    <t>NFM 6.3</t>
+    <t>Alk-IR</t>
+  </si>
+  <si>
+    <t>Alk-T-COL-BCG</t>
+  </si>
+  <si>
+    <t>Alk-T-COL-BCGMR</t>
+  </si>
+  <si>
+    <t>Alk-T-COL-MO</t>
+  </si>
+  <si>
+    <t>Alk-T-D1067-B</t>
+  </si>
+  <si>
+    <t>Alk-T-POT-Auto</t>
+  </si>
+  <si>
+    <t>Alk-T-POT-GRN</t>
+  </si>
+  <si>
+    <t>Alk-T-POT-PTC</t>
+  </si>
+  <si>
+    <t>Alk-T-POT-TE-Auto</t>
+  </si>
+  <si>
+    <t>Alk-T-POT-4.5-Auto</t>
+  </si>
+  <si>
+    <t>mg/l</t>
+  </si>
+  <si>
+    <t>me/L</t>
+  </si>
+  <si>
+    <t>Infrared Detection of CO2</t>
+  </si>
+  <si>
+    <t>Titration Method - Color Change using Bromcresol Green as Indicator (Endpoint pH=4.5)</t>
+  </si>
+  <si>
+    <t>Titration Method - Color Change using Bromcresol Green-Methyl Red as Indicator</t>
+  </si>
+  <si>
+    <t>Colorimetric Titration using Methyl Orange as Indicator (Endpoint pH=3.7)</t>
+  </si>
+  <si>
+    <t>Electrometric or Color-Change Titration</t>
+  </si>
+  <si>
+    <t>Potentiometric Titration using Titroprocessor (Endpoint not defined)</t>
+  </si>
+  <si>
+    <t>Gran Titration</t>
+  </si>
+  <si>
+    <t>Titration Method - Potentiometric Titration Curve</t>
+  </si>
+  <si>
+    <t>Two Endpoint Potentiometric Titration using Titroprocessor (Endpoints pH=4.5-4.2)</t>
+  </si>
+  <si>
+    <t>Titration Method - Potentiometric Titration to preselected pH using Titroprocessor (Endpoint pH=4.5)</t>
+  </si>
+  <si>
+    <t>Spectroscopy</t>
+  </si>
+  <si>
+    <t>Titration</t>
+  </si>
+  <si>
+    <t>Colorimetry</t>
+  </si>
+  <si>
+    <t>STAR 223</t>
+  </si>
+  <si>
+    <t>SM 2320 B4a</t>
+  </si>
+  <si>
+    <t>SM 403 4.a</t>
+  </si>
+  <si>
+    <t>D1067 B</t>
+  </si>
+  <si>
+    <t>ENV 373</t>
+  </si>
+  <si>
+    <t>ENV 372</t>
+  </si>
+  <si>
+    <t>SM 2320 B.4b</t>
+  </si>
+  <si>
+    <t>NAQ 10101</t>
+  </si>
+  <si>
+    <t>SM 2320 B4c</t>
   </si>
   <si>
     <t>Environment Canada 2007</t>
@@ -3921,22 +3972,46 @@
     <t>APHA 2012</t>
   </si>
   <si>
-    <t>USGS 1998</t>
-  </si>
-  <si>
-    <t>Specific Conductance of a solution is the ability of the solution to carry electric current and has some relationship to the Total Ionic Concentration of the solution. The sample temperature is brought to 20°C and the aliquot is measured electrometrically.</t>
-  </si>
-  <si>
-    <t>Specific conductance is measured in situ with a battery operated Conductivity-Temperature Meter, employing nickel electrodes in the four-electrode configuration with integral temperature sensor- compensator and internal calibration standards. The accuracy is ±2.5%.</t>
-  </si>
-  <si>
-    <t>Specific Conductance of a solution is the ability of the solution to carry electric current and has some relationship to the Total Ionic Concentration of the solution.~r~n The specific conductance is measured, using a radiometer CDM 83, automatic ranging conductivity meter and a radiometer type CDC 334 jacketed platinum electrode. A one-gallon water bath, with a HAAKE Model E52 temperature controller/circulation pump (or equivalent), accurately maintains the temperature bath at 25°C (± 0.1°C) and continually circulates water through the cell jacket. The sample aliquot is drawn into the conductivity cell via a vacuum and specific conductivity is read directly from the meter after a fifteen second temperature stabilization period. The radiometer is calibrated on a per use basis.~r~n The method detection limit is 0.2 µS/cm.~r~n 1 umho/cm = 1 µsie/cm. 1 µS/cm</t>
-  </si>
-  <si>
-    <t>Specific conductance is measured by a conductivity meter with Pt electrodes at the sample temperature (uncorrected).</t>
-  </si>
-  <si>
-    <t>In situ measurement generally is preferred for determining the conductivity of surface water; downhole or flowthrough-chamber measurements are preferred for ground water</t>
+    <t>APHA 1975</t>
+  </si>
+  <si>
+    <t>ASTM 1971</t>
+  </si>
+  <si>
+    <t>Environment Canada 1995</t>
+  </si>
+  <si>
+    <t>Environment Canada 1974</t>
+  </si>
+  <si>
+    <t>A filtered sample is mixed with HCl, then oxygen. The resulting CO2 is separated from the liquid phase and determined by in infrared detector.</t>
+  </si>
+  <si>
+    <t>A known volume of sample aliquot is titrated with standardized HCl to the end point colour change from blue to steel grey with a pH 4.5 indicator.</t>
+  </si>
+  <si>
+    <t>Alkalinity is defined as the quantitative capacity of a sample to neutralise a strong acid to a selected pH. A sample is preserved in the field at 4°C. If turbid, the sample is allowed to settle. A sample aliquot is titrated at 25°C, with standard H2SO4 using the mixed bromcresol green-methyl red indicator, and the colour response is indicated as follows: above pH 5.2, greenish blue; pH 5.0, light blue with lavender grey; pH 4.8, light-grey with bluish colour; and pH 4.6, light pink. The colour changes can be verified against a calibrated pH meter under the conditions of titratilon. An indicator blank is also titrated. The results are expressed as milliequivalents per litre of CaCO3.</t>
+  </si>
+  <si>
+    <t>(i) Mix 100 ml of sample with two or three drops of phenolphthalein indicator in a conical flask. (For determination of lower values of alkalinity use 200 ml of sample). (ii) If no colour change is produced, the alkalinity to phenolphthalein is zero. (iii) If the sample turns pink or red, determine the alkalinity to phenolphthalein by titration with standard acid (0.02N HCl) until the pink colour just disappears.(iv) In both cases (ii) and (iii) continue the determination using the sample to which phenolphthalein has been added.(v) Add a few drops of methyl orange indicator.(vi) If the sample turns orange without the addition of acid, the total alkalinity is zero.(vii) If the sample turns yellow, titrate with standard acid until the first perceptible colour change towards orange takes place.</t>
+  </si>
+  <si>
+    <t>A sample is preserved in the field at 4°C. If turbid, the sample is allowed to settle. A known volume of the sample aliquot is titrated with standardized H2SO4 or HCl to the methyl purple end point of pH=4.8 -5.4 calibrated for 25°C. Methyl purple indicator is used with a blue water-soluble dye to sharpen the end point. An indicator blank is also titrated. Alternatively, one can use methyl red indicator to a pH 4.8 end point [Japan method], or methyl red to a pH 5.4 end point [Russian method], or bromophenol blue measured colourimetrically at 600 nm [South Africa].</t>
+  </si>
+  <si>
+    <t>The total alkalinity is a measure of all hydroxides, carbonates and bicarbonates present in the water sample. Total alkalinity is determined in a whole water sample by potentiometric titration of a sample aliquot with a standard solution of sulphuric acid. This method employs an automated titrator which makes incremental additions of titrant to the sample and plots a titration curve. The titration curve is a plot of pH vs volume of titrant added. The endpoint of the titration is determined by analysis of the titration curve using a first derivative function to find the inflection point (curve changes from concave to convex or vice versa). The inflection point represents the stoichiometric equivalence point for the neutralization of the carbonates and other bases present. The total alkalinity is given by the equation F*X, where X= ml of acid needed to titrate to the inflection point and F is a factor derived from standardization of the acid. The factor F, incorporates the concentration of the acid used in the titration, the volume of sample analyzed and the conversion of the units to mg/L CaCO3.</t>
+  </si>
+  <si>
+    <t>The Gran Function employs an algorithm to determine inflection points from titration curves that are not well defined. The titration curves of low ionic strength soft waters and precipitation samples fall into this category. Total alkalinity of these samples is determined by titration with sulphuric acid employing an automatic titrator which makes incremental addition of titrant and plots a titration curve of pH against volume of titrant. Add 0.25mL 1 N KCl to 100mL of sample, then titrate to pH 3.7 with 0.001N HCl. ~r~n To use the Gran function, small increments of acid are added beyond the expected inflection point. Record both the incremental volumes added, and the corresponding pH. The volume corrected H+ concentration is plotted against the volume of added acid. The alkalinity is determined from extrapolation of the linear portion of the curve on the abscissa. Total alkalinity is given by the equation F*X, where X= ml of acid needed to titrate to the inflection point and F is a factor derived from standardization of the acid. The factor F incorporates the concentration of the acid used in the titration, the volume of sample analyzed, and the conversion of the units to mg/L CaCO3. The results of this titration, which is suitable only for very "soft" waters, may be either positive or negative.</t>
+  </si>
+  <si>
+    <t>Alkalinity is defined as the quantitative capacity of a sample to neutralise a strong acid to a selected pH. Select sample aliquot size (adjust to room temperature: 25°C) and normality of titrant. Add standard acid in increments of 0.5 mL or less, mix thoroughly; as the end point approaches, make smaller additions of acid and be sure the pH has reached equilibrium before adding more titrant. Titrate to pH of 3.7. Construct a titration curve by plotting the observed pH against the cumulative millilitres of titrant used. A smooth curve showing one or more inflections should be obtained (an erratic curve may indicate that equilibrium was not reached between successive additions). Results expressed as milliequivalent per litre of CaCO</t>
+  </si>
+  <si>
+    <t>Alkalinity is defined as the quantitative capacity of a sample to neutralise a strong acid to a selected pH. A sample is preserved in the field at 4°C. If turbid, the sample is allowed to settle. A known volume of the sample aliquot is titrated with a standardized solution of H2SO4 (or HCl), to pH=4.5 then to pH=4.2, using an automatic titrator and a pH meter calibrated for 25°C. The total alkalinity is found from both titration volumes. A two endpoint technique is employed to determine the actual inflection point.</t>
+  </si>
+  <si>
+    <t>If turbid, the sample is allowed to settle. An aliquot of the sample is then titrated with standard H2SO4 or HCL to pH 4.5 using an automatic titration system and a pH meter.</t>
   </si>
 </sst>
 </file>
@@ -14304,13 +14379,22 @@
         <v>1268</v>
       </c>
       <c r="C2" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="D2" t="s">
-        <v>1269</v>
+        <v>1270</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1271</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1272</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1273</v>
       </c>
       <c r="H2" t="s">
-        <v>1270</v>
+        <v>1274</v>
       </c>
     </row>
   </sheetData>
@@ -14320,7 +14404,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -14339,28 +14423,28 @@
         <v>1259</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1271</v>
+        <v>1275</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1272</v>
+        <v>1276</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1261</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>1273</v>
+        <v>1277</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>1274</v>
+        <v>1278</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1275</v>
+        <v>1279</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1276</v>
+        <v>1280</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>1277</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -14368,25 +14452,28 @@
         <v>1267</v>
       </c>
       <c r="B2" t="s">
-        <v>1278</v>
+        <v>1282</v>
       </c>
       <c r="C2" t="s">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="D2" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E2" t="s">
-        <v>1286</v>
+        <v>1294</v>
       </c>
       <c r="F2" t="s">
-        <v>1293</v>
+        <v>1304</v>
       </c>
       <c r="G2" t="s">
-        <v>1295</v>
+        <v>1307</v>
       </c>
       <c r="H2" t="s">
-        <v>1299</v>
+        <v>1316</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1322</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -14394,22 +14481,28 @@
         <v>1267</v>
       </c>
       <c r="B3" t="s">
-        <v>1279</v>
+        <v>1283</v>
       </c>
       <c r="C3" t="s">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="D3" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E3" t="s">
-        <v>1287</v>
+        <v>1295</v>
       </c>
       <c r="F3" t="s">
-        <v>1294</v>
+        <v>1305</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1308</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1317</v>
       </c>
       <c r="I3" t="s">
-        <v>1302</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -14417,19 +14510,28 @@
         <v>1267</v>
       </c>
       <c r="B4" t="s">
-        <v>1280</v>
+        <v>1284</v>
       </c>
       <c r="C4" t="s">
-        <v>1285</v>
+        <v>1293</v>
       </c>
       <c r="D4" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E4" t="s">
-        <v>1288</v>
+        <v>1296</v>
       </c>
       <c r="F4" t="s">
-        <v>1294</v>
+        <v>1305</v>
+      </c>
+      <c r="G4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="H4" t="s">
+        <v>1317</v>
+      </c>
+      <c r="I4" t="s">
+        <v>1324</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -14437,28 +14539,28 @@
         <v>1267</v>
       </c>
       <c r="B5" t="s">
-        <v>1281</v>
+        <v>1285</v>
       </c>
       <c r="C5" t="s">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="D5" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E5" t="s">
-        <v>1289</v>
+        <v>1297</v>
       </c>
       <c r="F5" t="s">
-        <v>1294</v>
+        <v>1306</v>
       </c>
       <c r="G5" t="s">
-        <v>1296</v>
+        <v>1309</v>
       </c>
       <c r="H5" t="s">
-        <v>1299</v>
+        <v>1318</v>
       </c>
       <c r="I5" t="s">
-        <v>1303</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -14466,28 +14568,28 @@
         <v>1267</v>
       </c>
       <c r="B6" t="s">
-        <v>1282</v>
+        <v>1286</v>
       </c>
       <c r="C6" t="s">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="D6" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E6" t="s">
-        <v>1290</v>
+        <v>1298</v>
       </c>
       <c r="F6" t="s">
-        <v>1294</v>
+        <v>1305</v>
       </c>
       <c r="G6" t="s">
-        <v>1297</v>
+        <v>1310</v>
       </c>
       <c r="H6" t="s">
-        <v>1300</v>
+        <v>1319</v>
       </c>
       <c r="I6" t="s">
-        <v>1304</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -14495,28 +14597,28 @@
         <v>1267</v>
       </c>
       <c r="B7" t="s">
-        <v>1283</v>
+        <v>1287</v>
       </c>
       <c r="C7" t="s">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="D7" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E7" t="s">
-        <v>1291</v>
+        <v>1299</v>
       </c>
       <c r="F7" t="s">
-        <v>1294</v>
+        <v>1305</v>
       </c>
       <c r="G7" t="s">
-        <v>1297</v>
+        <v>1311</v>
       </c>
       <c r="H7" t="s">
-        <v>1300</v>
+        <v>1320</v>
       </c>
       <c r="I7" t="s">
-        <v>1305</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -14524,28 +14626,115 @@
         <v>1267</v>
       </c>
       <c r="B8" t="s">
-        <v>1284</v>
+        <v>1288</v>
       </c>
       <c r="C8" t="s">
-        <v>1285</v>
+        <v>1292</v>
       </c>
       <c r="D8" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="E8" t="s">
+        <v>1300</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G8" t="s">
+        <v>1312</v>
+      </c>
+      <c r="H8" t="s">
+        <v>1320</v>
+      </c>
+      <c r="I8" t="s">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1293</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1301</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G9" t="s">
+        <v>1313</v>
+      </c>
+      <c r="H9" t="s">
+        <v>1317</v>
+      </c>
+      <c r="I9" t="s">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C10" t="s">
         <v>1292</v>
       </c>
-      <c r="F8" t="s">
-        <v>1294</v>
-      </c>
-      <c r="G8" t="s">
-        <v>1298</v>
-      </c>
-      <c r="H8" t="s">
-        <v>1301</v>
-      </c>
-      <c r="I8" t="s">
-        <v>1306</v>
+      <c r="D10" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G10" t="s">
+        <v>1314</v>
+      </c>
+      <c r="H10" t="s">
+        <v>1321</v>
+      </c>
+      <c r="I10" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1303</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1305</v>
+      </c>
+      <c r="G11" t="s">
+        <v>1315</v>
+      </c>
+      <c r="H11" t="s">
+        <v>1317</v>
+      </c>
+      <c r="I11" t="s">
+        <v>1331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
South African dissolved reactive phosphorus
</commit_message>
<xml_diff>
--- a/metadata.xlsx
+++ b/metadata.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2567" uniqueCount="1332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="1299">
   <si>
     <t>GEMS Station Number</t>
   </si>
@@ -3819,28 +3819,28 @@
     <t>Parameter Description</t>
   </si>
   <si>
-    <t>Alk-Tot</t>
-  </si>
-  <si>
-    <t>Alkalinity</t>
-  </si>
-  <si>
-    <t>Total Alkalinity</t>
-  </si>
-  <si>
-    <t>/Chemical/Inorganic/Non-Metal</t>
-  </si>
-  <si>
-    <t>207-439-9</t>
-  </si>
-  <si>
-    <t>471-34-1</t>
-  </si>
-  <si>
-    <t>3311</t>
-  </si>
-  <si>
-    <t>Acid-neutralizing capacity of sample at the point, when all Carbonate (CO32-) and Bicarbonate (HCO3-) have reacted, reported as mg CaCO3/L.</t>
+    <t>DRP</t>
+  </si>
+  <si>
+    <t>Orthophosphate</t>
+  </si>
+  <si>
+    <t>Dissolved Reactive Phosphorus</t>
+  </si>
+  <si>
+    <t>/Chemical/Nutrient/Phosphorous</t>
+  </si>
+  <si>
+    <t>604-302-9</t>
+  </si>
+  <si>
+    <t>14265-44-2</t>
+  </si>
+  <si>
+    <t>18367</t>
+  </si>
+  <si>
+    <t>Phosphate fractions in filtered samples responding to colorimetric tests without preliminary acid-hydrolysis or oxidative digestion (largely a measure of orthophosphates), reported as phosphorus.</t>
   </si>
   <si>
     <t>Analysis Method Code</t>
@@ -3864,154 +3864,55 @@
     <t>Method Description</t>
   </si>
   <si>
-    <t>Alk-IR</t>
-  </si>
-  <si>
-    <t>Alk-T-COL-BCG</t>
-  </si>
-  <si>
-    <t>Alk-T-COL-BCGMR</t>
-  </si>
-  <si>
-    <t>Alk-T-COL-MO</t>
-  </si>
-  <si>
-    <t>Alk-T-D1067-B</t>
-  </si>
-  <si>
-    <t>Alk-T-POT-Auto</t>
-  </si>
-  <si>
-    <t>Alk-T-POT-GRN</t>
-  </si>
-  <si>
-    <t>Alk-T-POT-PTC</t>
-  </si>
-  <si>
-    <t>Alk-T-POT-TE-Auto</t>
-  </si>
-  <si>
-    <t>Alk-T-POT-4.5-Auto</t>
+    <t>COL-AA</t>
+  </si>
+  <si>
+    <t>COL-SnCl</t>
+  </si>
+  <si>
+    <t>IC-CSC</t>
   </si>
   <si>
     <t>mg/l</t>
   </si>
   <si>
-    <t>me/L</t>
-  </si>
-  <si>
-    <t>Infrared Detection of CO2</t>
-  </si>
-  <si>
-    <t>Titration Method - Color Change using Bromcresol Green as Indicator (Endpoint pH=4.5)</t>
-  </si>
-  <si>
-    <t>Titration Method - Color Change using Bromcresol Green-Methyl Red as Indicator</t>
-  </si>
-  <si>
-    <t>Colorimetric Titration using Methyl Orange as Indicator (Endpoint pH=3.7)</t>
-  </si>
-  <si>
-    <t>Electrometric or Color-Change Titration</t>
-  </si>
-  <si>
-    <t>Potentiometric Titration using Titroprocessor (Endpoint not defined)</t>
-  </si>
-  <si>
-    <t>Gran Titration</t>
-  </si>
-  <si>
-    <t>Titration Method - Potentiometric Titration Curve</t>
-  </si>
-  <si>
-    <t>Two Endpoint Potentiometric Titration using Titroprocessor (Endpoints pH=4.5-4.2)</t>
-  </si>
-  <si>
-    <t>Titration Method - Potentiometric Titration to preselected pH using Titroprocessor (Endpoint pH=4.5)</t>
-  </si>
-  <si>
-    <t>Spectroscopy</t>
-  </si>
-  <si>
-    <t>Titration</t>
+    <t>Ascorbic Acid Method</t>
+  </si>
+  <si>
+    <t>Stannous Chloride Method</t>
+  </si>
+  <si>
+    <t>Ion Chromatography with Chemical Suppression of Eluent Conductivity</t>
   </si>
   <si>
     <t>Colorimetry</t>
   </si>
   <si>
-    <t>STAR 223</t>
-  </si>
-  <si>
-    <t>SM 2320 B4a</t>
-  </si>
-  <si>
-    <t>SM 403 4.a</t>
-  </si>
-  <si>
-    <t>D1067 B</t>
-  </si>
-  <si>
-    <t>ENV 373</t>
-  </si>
-  <si>
-    <t>ENV 372</t>
-  </si>
-  <si>
-    <t>SM 2320 B.4b</t>
-  </si>
-  <si>
-    <t>NAQ 10101</t>
-  </si>
-  <si>
-    <t>SM 2320 B4c</t>
-  </si>
-  <si>
-    <t>Environment Canada 2007</t>
+    <t>Chromatography</t>
+  </si>
+  <si>
+    <t>SM 4500-P E</t>
+  </si>
+  <si>
+    <t>SM 4500-P D</t>
+  </si>
+  <si>
+    <t>ISO 14911</t>
   </si>
   <si>
     <t>APHA 2012</t>
   </si>
   <si>
-    <t>APHA 1975</t>
-  </si>
-  <si>
-    <t>ASTM 1971</t>
-  </si>
-  <si>
-    <t>Environment Canada 1995</t>
-  </si>
-  <si>
-    <t>Environment Canada 1974</t>
-  </si>
-  <si>
-    <t>A filtered sample is mixed with HCl, then oxygen. The resulting CO2 is separated from the liquid phase and determined by in infrared detector.</t>
-  </si>
-  <si>
-    <t>A known volume of sample aliquot is titrated with standardized HCl to the end point colour change from blue to steel grey with a pH 4.5 indicator.</t>
-  </si>
-  <si>
-    <t>Alkalinity is defined as the quantitative capacity of a sample to neutralise a strong acid to a selected pH. A sample is preserved in the field at 4°C. If turbid, the sample is allowed to settle. A sample aliquot is titrated at 25°C, with standard H2SO4 using the mixed bromcresol green-methyl red indicator, and the colour response is indicated as follows: above pH 5.2, greenish blue; pH 5.0, light blue with lavender grey; pH 4.8, light-grey with bluish colour; and pH 4.6, light pink. The colour changes can be verified against a calibrated pH meter under the conditions of titratilon. An indicator blank is also titrated. The results are expressed as milliequivalents per litre of CaCO3.</t>
-  </si>
-  <si>
-    <t>(i) Mix 100 ml of sample with two or three drops of phenolphthalein indicator in a conical flask. (For determination of lower values of alkalinity use 200 ml of sample). (ii) If no colour change is produced, the alkalinity to phenolphthalein is zero. (iii) If the sample turns pink or red, determine the alkalinity to phenolphthalein by titration with standard acid (0.02N HCl) until the pink colour just disappears.(iv) In both cases (ii) and (iii) continue the determination using the sample to which phenolphthalein has been added.(v) Add a few drops of methyl orange indicator.(vi) If the sample turns orange without the addition of acid, the total alkalinity is zero.(vii) If the sample turns yellow, titrate with standard acid until the first perceptible colour change towards orange takes place.</t>
-  </si>
-  <si>
-    <t>A sample is preserved in the field at 4°C. If turbid, the sample is allowed to settle. A known volume of the sample aliquot is titrated with standardized H2SO4 or HCl to the methyl purple end point of pH=4.8 -5.4 calibrated for 25°C. Methyl purple indicator is used with a blue water-soluble dye to sharpen the end point. An indicator blank is also titrated. Alternatively, one can use methyl red indicator to a pH 4.8 end point [Japan method], or methyl red to a pH 5.4 end point [Russian method], or bromophenol blue measured colourimetrically at 600 nm [South Africa].</t>
-  </si>
-  <si>
-    <t>The total alkalinity is a measure of all hydroxides, carbonates and bicarbonates present in the water sample. Total alkalinity is determined in a whole water sample by potentiometric titration of a sample aliquot with a standard solution of sulphuric acid. This method employs an automated titrator which makes incremental additions of titrant to the sample and plots a titration curve. The titration curve is a plot of pH vs volume of titrant added. The endpoint of the titration is determined by analysis of the titration curve using a first derivative function to find the inflection point (curve changes from concave to convex or vice versa). The inflection point represents the stoichiometric equivalence point for the neutralization of the carbonates and other bases present. The total alkalinity is given by the equation F*X, where X= ml of acid needed to titrate to the inflection point and F is a factor derived from standardization of the acid. The factor F, incorporates the concentration of the acid used in the titration, the volume of sample analyzed and the conversion of the units to mg/L CaCO3.</t>
-  </si>
-  <si>
-    <t>The Gran Function employs an algorithm to determine inflection points from titration curves that are not well defined. The titration curves of low ionic strength soft waters and precipitation samples fall into this category. Total alkalinity of these samples is determined by titration with sulphuric acid employing an automatic titrator which makes incremental addition of titrant and plots a titration curve of pH against volume of titrant. Add 0.25mL 1 N KCl to 100mL of sample, then titrate to pH 3.7 with 0.001N HCl. ~r~n To use the Gran function, small increments of acid are added beyond the expected inflection point. Record both the incremental volumes added, and the corresponding pH. The volume corrected H+ concentration is plotted against the volume of added acid. The alkalinity is determined from extrapolation of the linear portion of the curve on the abscissa. Total alkalinity is given by the equation F*X, where X= ml of acid needed to titrate to the inflection point and F is a factor derived from standardization of the acid. The factor F incorporates the concentration of the acid used in the titration, the volume of sample analyzed, and the conversion of the units to mg/L CaCO3. The results of this titration, which is suitable only for very "soft" waters, may be either positive or negative.</t>
-  </si>
-  <si>
-    <t>Alkalinity is defined as the quantitative capacity of a sample to neutralise a strong acid to a selected pH. Select sample aliquot size (adjust to room temperature: 25°C) and normality of titrant. Add standard acid in increments of 0.5 mL or less, mix thoroughly; as the end point approaches, make smaller additions of acid and be sure the pH has reached equilibrium before adding more titrant. Titrate to pH of 3.7. Construct a titration curve by plotting the observed pH against the cumulative millilitres of titrant used. A smooth curve showing one or more inflections should be obtained (an erratic curve may indicate that equilibrium was not reached between successive additions). Results expressed as milliequivalent per litre of CaCO</t>
-  </si>
-  <si>
-    <t>Alkalinity is defined as the quantitative capacity of a sample to neutralise a strong acid to a selected pH. A sample is preserved in the field at 4°C. If turbid, the sample is allowed to settle. A known volume of the sample aliquot is titrated with a standardized solution of H2SO4 (or HCl), to pH=4.5 then to pH=4.2, using an automatic titrator and a pH meter calibrated for 25°C. The total alkalinity is found from both titration volumes. A two endpoint technique is employed to determine the actual inflection point.</t>
-  </si>
-  <si>
-    <t>If turbid, the sample is allowed to settle. An aliquot of the sample is then titrated with standard H2SO4 or HCL to pH 4.5 using an automatic titration system and a pH meter.</t>
+    <t>ISO 1998</t>
+  </si>
+  <si>
+    <t>Pipet 50.0mL sample into a test tube or 125mL Erlenmeyer flask. Add 0.05mL phenolphthalein indicator. If a red colour develops ad 5N H2SO4 solution dropwise to discharge the colour. Add 8.0mL combined reagent and mix thoroughly. After 10 min but no more than 30 min, measure absorbance of each sample at 880 nm, using reagent blank as the reference solution.</t>
+  </si>
+  <si>
+    <t>A sample is preserved in the field at 4°C (if not analysed immediately). The sample aliquot is mixed with ammonium molybdate to form the heteropoly molybdophosphoric acid and is reduced with stannous chloride, in an aqueous sulphuric acid medium, at 30°C, to form a molybdenum blue complex. The resulting blue colour is measured spectrometrically at 660 nm, and compared to identically-prepared PO4 standard and blank solutions. Interferences: Hg, at concentration of 1 mg/L, and As also interfere with the stannous chloride reagent.</t>
+  </si>
+  <si>
+    <t>A sample is filtered in the field through a 0.2 µm membrane filter. The sample aliquot is injected into an eluent stream, pumped through a separator column packed with anion exchange resin in the form of CO32-/HCO3-. The nitrate is separated, based on its affinity for the exchange sites of the resin bed. A suppressor reduces the background conductivity of the eluent and the concentration of phosphate is measured using a conductivity detector. The anion is identified by its retention time and its concentration by its peak height or area and compared to identically-prepared standard and blank solutions. Sample concentrations exceeding the linear range are diluted and re-run.</t>
   </si>
 </sst>
 </file>
@@ -14404,7 +14305,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="16.7109375" customWidth="1"/>
@@ -14455,25 +14356,25 @@
         <v>1282</v>
       </c>
       <c r="C2" t="s">
-        <v>1292</v>
+        <v>1285</v>
       </c>
       <c r="D2" t="s">
         <v>1269</v>
       </c>
       <c r="E2" t="s">
+        <v>1286</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1289</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="H2" t="s">
         <v>1294</v>
       </c>
-      <c r="F2" t="s">
-        <v>1304</v>
-      </c>
-      <c r="G2" t="s">
-        <v>1307</v>
-      </c>
-      <c r="H2" t="s">
-        <v>1316</v>
-      </c>
       <c r="I2" t="s">
-        <v>1322</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -14484,25 +14385,25 @@
         <v>1283</v>
       </c>
       <c r="C3" t="s">
-        <v>1292</v>
+        <v>1285</v>
       </c>
       <c r="D3" t="s">
         <v>1269</v>
       </c>
       <c r="E3" t="s">
-        <v>1295</v>
+        <v>1287</v>
       </c>
       <c r="F3" t="s">
-        <v>1305</v>
+        <v>1289</v>
       </c>
       <c r="G3" t="s">
-        <v>1308</v>
+        <v>1292</v>
       </c>
       <c r="H3" t="s">
-        <v>1317</v>
+        <v>1294</v>
       </c>
       <c r="I3" t="s">
-        <v>1323</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -14513,228 +14414,25 @@
         <v>1284</v>
       </c>
       <c r="C4" t="s">
-        <v>1293</v>
+        <v>1285</v>
       </c>
       <c r="D4" t="s">
         <v>1269</v>
       </c>
       <c r="E4" t="s">
-        <v>1296</v>
+        <v>1288</v>
       </c>
       <c r="F4" t="s">
-        <v>1305</v>
+        <v>1290</v>
       </c>
       <c r="G4" t="s">
-        <v>1308</v>
+        <v>1293</v>
       </c>
       <c r="H4" t="s">
-        <v>1317</v>
+        <v>1295</v>
       </c>
       <c r="I4" t="s">
-        <v>1324</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1285</v>
-      </c>
-      <c r="C5" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E5" t="s">
-        <v>1297</v>
-      </c>
-      <c r="F5" t="s">
-        <v>1306</v>
-      </c>
-      <c r="G5" t="s">
-        <v>1309</v>
-      </c>
-      <c r="H5" t="s">
-        <v>1318</v>
-      </c>
-      <c r="I5" t="s">
-        <v>1325</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1286</v>
-      </c>
-      <c r="C6" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D6" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E6" t="s">
         <v>1298</v>
-      </c>
-      <c r="F6" t="s">
-        <v>1305</v>
-      </c>
-      <c r="G6" t="s">
-        <v>1310</v>
-      </c>
-      <c r="H6" t="s">
-        <v>1319</v>
-      </c>
-      <c r="I6" t="s">
-        <v>1326</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1287</v>
-      </c>
-      <c r="C7" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E7" t="s">
-        <v>1299</v>
-      </c>
-      <c r="F7" t="s">
-        <v>1305</v>
-      </c>
-      <c r="G7" t="s">
-        <v>1311</v>
-      </c>
-      <c r="H7" t="s">
-        <v>1320</v>
-      </c>
-      <c r="I7" t="s">
-        <v>1327</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1288</v>
-      </c>
-      <c r="C8" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D8" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E8" t="s">
-        <v>1300</v>
-      </c>
-      <c r="F8" t="s">
-        <v>1305</v>
-      </c>
-      <c r="G8" t="s">
-        <v>1312</v>
-      </c>
-      <c r="H8" t="s">
-        <v>1320</v>
-      </c>
-      <c r="I8" t="s">
-        <v>1328</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B9" t="s">
-        <v>1289</v>
-      </c>
-      <c r="C9" t="s">
-        <v>1293</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E9" t="s">
-        <v>1301</v>
-      </c>
-      <c r="F9" t="s">
-        <v>1305</v>
-      </c>
-      <c r="G9" t="s">
-        <v>1313</v>
-      </c>
-      <c r="H9" t="s">
-        <v>1317</v>
-      </c>
-      <c r="I9" t="s">
-        <v>1329</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B10" t="s">
-        <v>1290</v>
-      </c>
-      <c r="C10" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E10" t="s">
-        <v>1302</v>
-      </c>
-      <c r="F10" t="s">
-        <v>1305</v>
-      </c>
-      <c r="G10" t="s">
-        <v>1314</v>
-      </c>
-      <c r="H10" t="s">
-        <v>1321</v>
-      </c>
-      <c r="I10" t="s">
-        <v>1330</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
-        <v>1267</v>
-      </c>
-      <c r="B11" t="s">
-        <v>1291</v>
-      </c>
-      <c r="C11" t="s">
-        <v>1292</v>
-      </c>
-      <c r="D11" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E11" t="s">
-        <v>1303</v>
-      </c>
-      <c r="F11" t="s">
-        <v>1305</v>
-      </c>
-      <c r="G11" t="s">
-        <v>1315</v>
-      </c>
-      <c r="H11" t="s">
-        <v>1317</v>
-      </c>
-      <c r="I11" t="s">
-        <v>1331</v>
       </c>
     </row>
   </sheetData>

</xml_diff>